<commit_message>
Aquí m'he tornat boig, canvis a dojo!!!!
--HG--
branch : Proves PiG
</commit_message>
<xml_diff>
--- a/Docs/Arcelor-Moviments.xlsx
+++ b/Docs/Arcelor-Moviments.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Repositoris\C#\_Actiu\InversionsV2\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{148F13AB-688F-408A-95AF-F3ED5A4BEC99}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8FF1D927-3846-4923-A602-60020A4C88B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{3BE38316-2729-4F6D-9D30-9A2EA6E3D00C}"/>
+    <workbookView xWindow="22932" yWindow="0" windowWidth="23256" windowHeight="12576" xr2:uid="{3BE38316-2729-4F6D-9D30-9A2EA6E3D00C}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="10">
   <si>
     <t>Compra</t>
   </si>
@@ -50,13 +50,20 @@
   <si>
     <t>Desp</t>
   </si>
+  <si>
+    <t>Dividents per compra</t>
+  </si>
+  <si>
+    <t>Parts per càlcul divid</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="8" formatCode="#,##0.00\ &quot;€&quot;;[Red]\-#,##0.00\ &quot;€&quot;"/>
+    <numFmt numFmtId="164" formatCode="#,##0.000\ &quot;€&quot;;[Red]\-#,##0.000\ &quot;€&quot;"/>
   </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
@@ -75,12 +82,24 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -95,7 +114,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -114,6 +133,25 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="8" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="3" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -429,16 +467,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4AB00EBE-D099-434F-AF7E-F7D80ABD81FB}">
-  <dimension ref="A1:H38"/>
+  <dimension ref="A1:M38"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="5" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="10" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="10.7265625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="2" customWidth="1"/>
+    <col min="8" max="8" width="9.90625" style="16" customWidth="1"/>
+    <col min="9" max="9" width="11.36328125" customWidth="1"/>
+    <col min="10" max="10" width="11.26953125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:13" ht="29" x14ac:dyDescent="0.35">
       <c r="D1" s="5" t="s">
         <v>4</v>
       </c>
@@ -449,11 +490,17 @@
         <v>7</v>
       </c>
       <c r="G1" s="5"/>
-      <c r="H1" s="6" t="s">
+      <c r="H1" s="15" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I1" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="J1" s="6" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A2" s="1">
         <v>79</v>
       </c>
@@ -473,12 +520,12 @@
         <v>15.06</v>
       </c>
       <c r="G2" s="3"/>
-      <c r="H2">
+      <c r="H2" s="16">
         <f>D2</f>
         <v>925</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A3" s="1">
         <v>80</v>
       </c>
@@ -498,12 +545,12 @@
         <v>25.32</v>
       </c>
       <c r="G3" s="3"/>
-      <c r="H3">
+      <c r="H3" s="16">
         <f>H2-D3</f>
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A4" s="1">
         <v>81</v>
       </c>
@@ -523,12 +570,12 @@
         <v>15.06</v>
       </c>
       <c r="G4" s="3"/>
-      <c r="H4">
+      <c r="H4" s="16">
         <f>H3+D4</f>
         <v>929</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A5" s="1">
         <v>82</v>
       </c>
@@ -548,12 +595,12 @@
         <v>15.09</v>
       </c>
       <c r="G5" s="3"/>
-      <c r="H5">
+      <c r="H5" s="16">
         <f>H4-D5</f>
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A6" s="1">
         <v>83</v>
       </c>
@@ -573,12 +620,12 @@
         <v>20.14</v>
       </c>
       <c r="G6" s="3"/>
-      <c r="H6">
+      <c r="H6" s="16">
         <f t="shared" ref="H6:H37" si="0">H5+D6</f>
         <v>5386</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A7" s="1">
         <v>84</v>
       </c>
@@ -598,12 +645,12 @@
         <v>20.03</v>
       </c>
       <c r="G7" s="3"/>
-      <c r="H7">
+      <c r="H7" s="16">
         <f>H6-D7</f>
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A8" s="1">
         <v>94</v>
       </c>
@@ -623,12 +670,12 @@
         <v>20.149999999999999</v>
       </c>
       <c r="G8" s="3"/>
-      <c r="H8">
+      <c r="H8" s="16">
         <f t="shared" si="0"/>
         <v>6415</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A9" s="1">
         <v>97</v>
       </c>
@@ -648,12 +695,12 @@
         <v>20.399999999999999</v>
       </c>
       <c r="G9" s="3"/>
-      <c r="H9">
+      <c r="H9" s="16">
         <f>H8-D9</f>
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A10" s="1">
         <v>138</v>
       </c>
@@ -673,11 +720,11 @@
         <v>0</v>
       </c>
       <c r="G10" s="3"/>
-      <c r="H10">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="H10" s="16">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A11" s="1">
         <v>151</v>
       </c>
@@ -697,12 +744,12 @@
         <v>15.15</v>
       </c>
       <c r="G11" s="3"/>
-      <c r="H11">
+      <c r="H11" s="16">
         <f t="shared" si="0"/>
         <v>527</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A12" s="1">
         <v>165</v>
       </c>
@@ -722,16 +769,16 @@
         <v>27.45</v>
       </c>
       <c r="G12" s="3"/>
-      <c r="H12">
+      <c r="H12" s="16">
         <f>H11-D12</f>
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A13" s="1">
         <v>166</v>
       </c>
-      <c r="B13" s="1" t="s">
+      <c r="B13" s="8" t="s">
         <v>0</v>
       </c>
       <c r="C13" s="2">
@@ -747,12 +794,20 @@
         <v>28.51</v>
       </c>
       <c r="G13" s="1"/>
-      <c r="H13" s="1">
+      <c r="H13" s="17">
         <f t="shared" si="0"/>
         <v>1600</v>
       </c>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I13" s="9">
+        <f>D13-D14</f>
+        <v>952</v>
+      </c>
+      <c r="J13" s="12">
+        <f>E$16/H$16*I13</f>
+        <v>169.60813559322034</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A14" s="1">
         <v>169</v>
       </c>
@@ -772,16 +827,17 @@
         <v>10.06</v>
       </c>
       <c r="G14" s="1"/>
-      <c r="H14" s="1">
+      <c r="H14" s="17">
         <f>H13-D14</f>
         <v>952</v>
       </c>
-    </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="J14" s="13"/>
+    </row>
+    <row r="15" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A15" s="1">
         <v>174</v>
       </c>
-      <c r="B15" s="1" t="s">
+      <c r="B15" s="8" t="s">
         <v>0</v>
       </c>
       <c r="C15" s="2">
@@ -797,16 +853,36 @@
         <v>10.06</v>
       </c>
       <c r="G15" s="1"/>
-      <c r="H15" s="1">
+      <c r="H15" s="17">
         <f t="shared" si="0"/>
         <v>1652</v>
       </c>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I15" s="9">
+        <f>D15</f>
+        <v>700</v>
+      </c>
+      <c r="J15" s="12">
+        <f>E$16/H$16*I15</f>
+        <v>124.71186440677965</v>
+      </c>
+      <c r="K15">
+        <f>H17</f>
+        <v>400</v>
+      </c>
+      <c r="L15" s="13">
+        <f>J15/D15*K15</f>
+        <v>71.263922518159802</v>
+      </c>
+      <c r="M15" s="7">
+        <f>F15/D15*K15</f>
+        <v>5.7485714285714282</v>
+      </c>
+    </row>
+    <row r="16" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A16" s="1">
         <v>176</v>
       </c>
-      <c r="B16" s="1" t="s">
+      <c r="B16" s="8" t="s">
         <v>1</v>
       </c>
       <c r="C16" s="2">
@@ -822,12 +898,13 @@
         <v>0</v>
       </c>
       <c r="G16" s="1"/>
-      <c r="H16" s="1">
+      <c r="H16" s="17">
         <f t="shared" si="0"/>
         <v>1652</v>
       </c>
-    </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="J16" s="13"/>
+    </row>
+    <row r="17" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A17" s="1">
         <v>177</v>
       </c>
@@ -847,12 +924,13 @@
         <v>10.06</v>
       </c>
       <c r="G17" s="1"/>
-      <c r="H17" s="1">
+      <c r="H17" s="17">
         <f>H16-D17</f>
         <v>400</v>
       </c>
-    </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="J17" s="13"/>
+    </row>
+    <row r="18" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A18" s="1">
         <v>178</v>
       </c>
@@ -872,16 +950,19 @@
         <v>10.06</v>
       </c>
       <c r="G18" s="1"/>
-      <c r="H18" s="1">
+      <c r="H18" s="17">
         <f>H17+D18</f>
         <v>900</v>
       </c>
-    </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="J18" s="13"/>
+      <c r="L18" s="13"/>
+      <c r="M18" s="7"/>
+    </row>
+    <row r="19" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A19" s="1">
         <v>191</v>
       </c>
-      <c r="B19" s="1" t="s">
+      <c r="B19" s="10" t="s">
         <v>0</v>
       </c>
       <c r="C19" s="2">
@@ -897,12 +978,22 @@
         <v>10.17</v>
       </c>
       <c r="G19" s="1"/>
-      <c r="H19" s="1">
-        <f>H18+D19</f>
+      <c r="H19" s="17">
+        <f t="shared" ref="H19:H24" si="1">H18+D19</f>
         <v>1560</v>
       </c>
-    </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I19" s="10">
+        <f>H21</f>
+        <v>400</v>
+      </c>
+      <c r="J19" s="14">
+        <f>E$25/H$25*I19</f>
+        <v>98.351578947368424</v>
+      </c>
+      <c r="L19" s="13"/>
+      <c r="M19" s="7"/>
+    </row>
+    <row r="20" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A20" s="1">
         <v>190</v>
       </c>
@@ -922,12 +1013,15 @@
         <v>5.0599999999999996</v>
       </c>
       <c r="G20" s="1"/>
-      <c r="H20" s="1">
-        <f t="shared" si="0"/>
+      <c r="H20" s="17">
+        <f t="shared" si="1"/>
         <v>1652</v>
       </c>
-    </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="J20" s="13"/>
+      <c r="L20" s="13"/>
+      <c r="M20" s="7"/>
+    </row>
+    <row r="21" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A21" s="1">
         <v>179</v>
       </c>
@@ -947,16 +1041,19 @@
         <v>16.54</v>
       </c>
       <c r="G21" s="1"/>
-      <c r="H21" s="1">
+      <c r="H21" s="17">
         <f>H20-D21</f>
         <v>400</v>
       </c>
-    </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="J21" s="13"/>
+      <c r="L21" s="13"/>
+      <c r="M21" s="13"/>
+    </row>
+    <row r="22" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A22" s="1">
         <v>193</v>
       </c>
-      <c r="B22" s="1" t="s">
+      <c r="B22" s="10" t="s">
         <v>0</v>
       </c>
       <c r="C22" s="2">
@@ -972,16 +1069,24 @@
         <v>8.06</v>
       </c>
       <c r="G22" s="1"/>
-      <c r="H22" s="1">
-        <f t="shared" si="0"/>
+      <c r="H22" s="17">
+        <f t="shared" si="1"/>
         <v>833</v>
       </c>
-    </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I22" s="11">
+        <f>D22</f>
+        <v>433</v>
+      </c>
+      <c r="J22" s="14">
+        <f>E$25/H$25*I22</f>
+        <v>106.46558421052632</v>
+      </c>
+    </row>
+    <row r="23" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A23" s="1">
         <v>192</v>
       </c>
-      <c r="B23" s="1" t="s">
+      <c r="B23" s="10" t="s">
         <v>0</v>
       </c>
       <c r="C23" s="2">
@@ -997,16 +1102,24 @@
         <v>10.06</v>
       </c>
       <c r="G23" s="1"/>
-      <c r="H23" s="1">
-        <f t="shared" si="0"/>
+      <c r="H23" s="17">
+        <f t="shared" si="1"/>
         <v>1333</v>
       </c>
-    </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I23" s="11">
+        <f>D23</f>
+        <v>500</v>
+      </c>
+      <c r="J23" s="14">
+        <f>E$25/H$25*I23</f>
+        <v>122.93947368421053</v>
+      </c>
+    </row>
+    <row r="24" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A24" s="1">
         <v>182</v>
       </c>
-      <c r="B24" s="1" t="s">
+      <c r="B24" s="10" t="s">
         <v>0</v>
       </c>
       <c r="C24" s="2">
@@ -1022,16 +1135,24 @@
         <v>10.17</v>
       </c>
       <c r="G24" s="1"/>
-      <c r="H24" s="1">
-        <f t="shared" si="0"/>
+      <c r="H24" s="17">
+        <f t="shared" si="1"/>
         <v>1900</v>
       </c>
-    </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I24" s="11">
+        <f>D24</f>
+        <v>567</v>
+      </c>
+      <c r="J24" s="14">
+        <f>E$25/H$25*I24</f>
+        <v>139.41336315789474</v>
+      </c>
+    </row>
+    <row r="25" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A25" s="1">
         <v>195</v>
       </c>
-      <c r="B25" s="1" t="s">
+      <c r="B25" s="10" t="s">
         <v>1</v>
       </c>
       <c r="C25" s="2">
@@ -1047,12 +1168,13 @@
         <v>0</v>
       </c>
       <c r="G25" s="1"/>
-      <c r="H25" s="1">
-        <f t="shared" si="0"/>
+      <c r="H25" s="17">
+        <f>H24+D25</f>
         <v>1900</v>
       </c>
-    </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="J25" s="7"/>
+    </row>
+    <row r="26" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A26" s="1">
         <v>206</v>
       </c>
@@ -1072,12 +1194,12 @@
         <v>0.61</v>
       </c>
       <c r="G26" s="1"/>
-      <c r="H26" s="1">
-        <f t="shared" ref="H26:H35" si="1">H25-D26</f>
+      <c r="H26" s="17">
+        <f>H25-D26</f>
         <v>1846</v>
       </c>
     </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A27" s="1">
         <v>207</v>
       </c>
@@ -1097,12 +1219,12 @@
         <v>9.56</v>
       </c>
       <c r="G27" s="1"/>
-      <c r="H27" s="1">
-        <f t="shared" si="1"/>
+      <c r="H27" s="17">
+        <f t="shared" ref="H27:H35" si="2">H26-D27</f>
         <v>1000</v>
       </c>
     </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A28" s="1">
         <v>208</v>
       </c>
@@ -1122,12 +1244,12 @@
         <v>0.3</v>
       </c>
       <c r="G28" s="1"/>
-      <c r="H28" s="1">
-        <f t="shared" si="1"/>
+      <c r="H28" s="17">
+        <f t="shared" si="2"/>
         <v>972</v>
       </c>
     </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A29" s="1">
         <v>209</v>
       </c>
@@ -1147,12 +1269,12 @@
         <v>0.48</v>
       </c>
       <c r="G29" s="1"/>
-      <c r="H29" s="1">
-        <f t="shared" si="1"/>
+      <c r="H29" s="17">
+        <f t="shared" si="2"/>
         <v>928</v>
       </c>
     </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A30" s="1">
         <v>210</v>
       </c>
@@ -1172,12 +1294,12 @@
         <v>0.31</v>
       </c>
       <c r="G30" s="3"/>
-      <c r="H30">
-        <f t="shared" si="1"/>
+      <c r="H30" s="16">
+        <f t="shared" si="2"/>
         <v>899</v>
       </c>
     </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A31" s="1">
         <v>211</v>
       </c>
@@ -1197,12 +1319,12 @@
         <v>0.91</v>
       </c>
       <c r="G31" s="3"/>
-      <c r="H31">
-        <f t="shared" si="1"/>
+      <c r="H31" s="16">
+        <f t="shared" si="2"/>
         <v>815</v>
       </c>
     </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A32" s="1">
         <v>212</v>
       </c>
@@ -1222,8 +1344,8 @@
         <v>1.63</v>
       </c>
       <c r="G32" s="3"/>
-      <c r="H32">
-        <f t="shared" si="1"/>
+      <c r="H32" s="16">
+        <f t="shared" si="2"/>
         <v>665</v>
       </c>
     </row>
@@ -1247,8 +1369,8 @@
         <v>4.84</v>
       </c>
       <c r="G33" s="3"/>
-      <c r="H33">
-        <f t="shared" si="1"/>
+      <c r="H33" s="16">
+        <f t="shared" si="2"/>
         <v>218</v>
       </c>
     </row>
@@ -1272,8 +1394,8 @@
         <v>0.78</v>
       </c>
       <c r="G34" s="3"/>
-      <c r="H34">
-        <f t="shared" si="1"/>
+      <c r="H34" s="16">
+        <f t="shared" si="2"/>
         <v>146</v>
       </c>
     </row>
@@ -1297,8 +1419,8 @@
         <v>1.58</v>
       </c>
       <c r="G35" s="3"/>
-      <c r="H35">
-        <f t="shared" si="1"/>
+      <c r="H35" s="16">
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -1322,7 +1444,7 @@
         <v>11.4</v>
       </c>
       <c r="G36" s="3"/>
-      <c r="H36">
+      <c r="H36" s="16">
         <f t="shared" si="0"/>
         <v>579</v>
       </c>
@@ -1347,7 +1469,7 @@
         <v>8.1</v>
       </c>
       <c r="G37" s="3"/>
-      <c r="H37">
+      <c r="H37" s="16">
         <f t="shared" si="0"/>
         <v>990</v>
       </c>
@@ -1372,7 +1494,7 @@
         <v>9.89</v>
       </c>
       <c r="G38" s="3"/>
-      <c r="H38">
+      <c r="H38" s="16">
         <f>H37-D38</f>
         <v>0</v>
       </c>

</xml_diff>